<commit_message>
base tickers atualizada 10-09
</commit_message>
<xml_diff>
--- a/lista_tickers_liquidos.xlsx
+++ b/lista_tickers_liquidos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GiovanniAzevedoCharr\Documents\python_projects\Robust_decisor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GiovanniAzevedoCharr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8B1815-2284-404C-9CF1-A08B81AD0ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B1566D-ECD7-4847-8C83-D7CD9E0432E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>ticker</t>
   </si>
@@ -34,9 +34,6 @@
     <t>ASAI3</t>
   </si>
   <si>
-    <t>AURE3</t>
-  </si>
-  <si>
     <t>AZZA3</t>
   </si>
   <si>
@@ -181,9 +178,6 @@
     <t>RDOR3</t>
   </si>
   <si>
-    <t>RECV3</t>
-  </si>
-  <si>
     <t>RENT3</t>
   </si>
   <si>
@@ -193,9 +187,6 @@
     <t>SBSP3</t>
   </si>
   <si>
-    <t>SLCE3</t>
-  </si>
-  <si>
     <t>SMFT3</t>
   </si>
   <si>
@@ -241,9 +232,6 @@
     <t>AXIA3</t>
   </si>
   <si>
-    <t>AXIA6</t>
-  </si>
-  <si>
     <t>CEAB3</t>
   </si>
   <si>
@@ -260,6 +248,81 @@
   </si>
   <si>
     <t>MBRF3</t>
+  </si>
+  <si>
+    <t>BOVA11</t>
+  </si>
+  <si>
+    <t>SMAL11</t>
+  </si>
+  <si>
+    <t>IBOV11</t>
+  </si>
+  <si>
+    <t>ROXO34</t>
+  </si>
+  <si>
+    <t>LWSA3</t>
+  </si>
+  <si>
+    <t>SIMH3</t>
+  </si>
+  <si>
+    <t>MOVI3</t>
+  </si>
+  <si>
+    <t>IRBR3</t>
+  </si>
+  <si>
+    <t>JHSF3</t>
+  </si>
+  <si>
+    <t>SAPR11</t>
+  </si>
+  <si>
+    <t>AUAU3</t>
+  </si>
+  <si>
+    <t>VULC3</t>
+  </si>
+  <si>
+    <t>ANIM3</t>
+  </si>
+  <si>
+    <t>EZTC3</t>
+  </si>
+  <si>
+    <t>CVCB3</t>
+  </si>
+  <si>
+    <t>TEND3</t>
+  </si>
+  <si>
+    <t>RAPT4</t>
+  </si>
+  <si>
+    <t>TASA4</t>
+  </si>
+  <si>
+    <t>BRSR6</t>
+  </si>
+  <si>
+    <t>BHIA3</t>
+  </si>
+  <si>
+    <t>RAIZ4</t>
+  </si>
+  <si>
+    <t>XPBR31</t>
+  </si>
+  <si>
+    <t>ALPA4</t>
+  </si>
+  <si>
+    <t>ECOR3</t>
+  </si>
+  <si>
+    <t>SAUD3</t>
   </si>
 </sst>
 </file>
@@ -277,12 +340,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -538,7 +603,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:A80"/>
+  <dimension ref="A1:A101"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
@@ -548,327 +613,327 @@
     </row>
     <row r="2" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>72</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>73</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>74</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>43</v>
+        <v>12</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>52</v>
+        <v>16</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>54</v>
+        <v>84</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="15" x14ac:dyDescent="0.25">
@@ -878,67 +943,172 @@
     </row>
     <row r="68" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>59</v>
+        <v>87</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="75" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
     </row>
     <row r="76" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
     </row>
     <row r="77" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>68</v>
+        <v>34</v>
       </c>
     </row>
     <row r="78" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="80" spans="1:1" ht="15" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>71</v>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>